<commit_message>
feat(2026-06-06): update Kahoot questions and import sheet
</commit_message>
<xml_diff>
--- a/2026-06-06_Agentic_AI_Mission_Control/2026-06-06_Kahoot_Import.xlsx
+++ b/2026-06-06_Agentic_AI_Mission_Control/2026-06-06_Kahoot_Import.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G16"/>
+  <dimension ref="A1:G19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -948,6 +948,105 @@
         <v>1</v>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>According to the "How We Got Here" slide, what happened in November 2022?</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>ChatGPT made an AI chat interface become mainstream</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Claude Code became a coding agent in the terminal</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Operator became a browser agent for web tasks</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>OpenClaw and Hermes connected models to tools</t>
+        </is>
+      </c>
+      <c r="F17" t="n">
+        <v>25</v>
+      </c>
+      <c r="G17" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>On the timeline, what did GPT-4 and Claude represent in March 2023?</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Stronger reasoning assistants</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Apps that no longer need testing</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>A rule that agents should delete files</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>A tool only for typing practice</t>
+        </is>
+      </c>
+      <c r="F18" t="n">
+        <v>25</v>
+      </c>
+      <c r="G18" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>What is the main trend shown from ChatGPT to Codex and 2026 agent platforms?</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>AI tools are moving from chat toward using tools with human supervision</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>AI stopped using language</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Humans no longer need to set limits</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Testing became unnecessary</t>
+        </is>
+      </c>
+      <c r="F19" t="n">
+        <v>25</v>
+      </c>
+      <c r="G19" t="n">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>